<commit_message>
data: cierre dia 2026-08-31_2001 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/Plan cobertura/on premise.xlsx
+++ b/01_INPUTS/Plan cobertura/on premise.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Orbit\MATINAL_PENAFLOR\01_INPUTS\Plan cobertura\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E72926B-255E-46B0-8427-10A14B84B28D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A86DDA83-D565-4CD9-86BE-7607B82286DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{BDD19824-CB24-4B71-8F29-D0B48A768086}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{BDD19824-CB24-4B71-8F29-D0B48A768086}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2377" uniqueCount="784">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2378" uniqueCount="785">
   <si>
     <t>INFORMACIÓN DEL PUNTO DE VENTA</t>
   </si>
@@ -2390,6 +2390,9 @@
   </si>
   <si>
     <t>Grupo Ronda</t>
+  </si>
+  <si>
+    <t>Salagre</t>
   </si>
 </sst>
 </file>
@@ -2557,13 +2560,13 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2897,16 +2900,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
       <c r="I1" s="1" t="s">
         <v>1</v>
       </c>
@@ -26290,14 +26293,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{187DECAE-1233-4914-9737-66C0131BABF4}">
-  <dimension ref="B1:D12"/>
+  <dimension ref="B1:D13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="11.42578125" style="17"/>
+    <col min="2" max="2" width="11.42578125" style="15"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="15" t="s">
         <v>772</v>
       </c>
       <c r="C1" t="s">
@@ -26308,7 +26311,7 @@
       </c>
     </row>
     <row r="2" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B2" s="17">
+      <c r="B2" s="15">
         <v>1409</v>
       </c>
       <c r="C2" t="s">
@@ -26319,7 +26322,7 @@
       </c>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B3" s="17">
+      <c r="B3" s="15">
         <v>1371</v>
       </c>
       <c r="C3" t="s">
@@ -26330,7 +26333,7 @@
       </c>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B4" s="17">
+      <c r="B4" s="15">
         <v>1425</v>
       </c>
       <c r="C4" t="s">
@@ -26341,7 +26344,7 @@
       </c>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B5" s="17">
+      <c r="B5" s="15">
         <v>1408</v>
       </c>
       <c r="C5" t="s">
@@ -26352,7 +26355,7 @@
       </c>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B6" s="17">
+      <c r="B6" s="15">
         <v>1410</v>
       </c>
       <c r="C6" t="s">
@@ -26363,7 +26366,7 @@
       </c>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B7" s="17">
+      <c r="B7" s="15">
         <v>1446</v>
       </c>
       <c r="C7" t="s">
@@ -26374,7 +26377,7 @@
       </c>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B8" s="17">
+      <c r="B8" s="15">
         <v>1400</v>
       </c>
       <c r="C8" t="s">
@@ -26385,7 +26388,7 @@
       </c>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B9" s="17">
+      <c r="B9" s="15">
         <v>1407</v>
       </c>
       <c r="C9" t="s">
@@ -26396,7 +26399,7 @@
       </c>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B10" s="17">
+      <c r="B10" s="15">
         <v>1437</v>
       </c>
       <c r="C10" t="s">
@@ -26407,7 +26410,7 @@
       </c>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B11" s="17">
+      <c r="B11" s="15">
         <v>1428</v>
       </c>
       <c r="C11" t="s">
@@ -26418,7 +26421,7 @@
       </c>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B12" s="17">
+      <c r="B12" s="15">
         <v>1368</v>
       </c>
       <c r="C12" t="s">
@@ -26426,6 +26429,17 @@
       </c>
       <c r="D12">
         <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B13" s="15">
+        <v>1476</v>
+      </c>
+      <c r="C13" t="s">
+        <v>784</v>
+      </c>
+      <c r="D13">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: cierre dia 2026-09-10_1906 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/Plan cobertura/on premise.xlsx
+++ b/01_INPUTS/Plan cobertura/on premise.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Orbit\MATINAL_PENAFLOR\01_INPUTS\Plan cobertura\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A86DDA83-D565-4CD9-86BE-7607B82286DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40E79592-6E00-4334-8C72-FEFF807E0CE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{BDD19824-CB24-4B71-8F29-D0B48A768086}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2378" uniqueCount="785">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2380" uniqueCount="787">
   <si>
     <t>INFORMACIÓN DEL PUNTO DE VENTA</t>
   </si>
@@ -2393,6 +2393,12 @@
   </si>
   <si>
     <t>Salagre</t>
+  </si>
+  <si>
+    <t>Svetac Ariel</t>
+  </si>
+  <si>
+    <t>alta ganada</t>
   </si>
 </sst>
 </file>
@@ -7844,9 +7850,11 @@
       <c r="L97" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="M97" s="9"/>
+      <c r="M97" s="9">
+        <v>1482</v>
+      </c>
       <c r="N97" s="9" t="s">
-        <v>33</v>
+        <v>786</v>
       </c>
       <c r="O97" s="3"/>
       <c r="P97" s="3"/>
@@ -9748,8 +9756,12 @@
       <c r="L134" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="M134" s="9"/>
-      <c r="N134" s="9"/>
+      <c r="M134" s="9">
+        <v>1484</v>
+      </c>
+      <c r="N134" s="9" t="s">
+        <v>786</v>
+      </c>
       <c r="O134" s="3"/>
       <c r="P134" s="3"/>
       <c r="Q134" s="3"/>
@@ -26293,7 +26305,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{187DECAE-1233-4914-9737-66C0131BABF4}">
-  <dimension ref="B1:D13"/>
+  <dimension ref="B1:D14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="11.42578125" style="15"/>
@@ -26442,6 +26454,17 @@
         <v>9</v>
       </c>
     </row>
+    <row r="14" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B14" s="15">
+        <v>1479</v>
+      </c>
+      <c r="C14" t="s">
+        <v>785</v>
+      </c>
+      <c r="D14">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>